<commit_message>
let the classification step pick S2's top features once, not twice with different tie rules
</commit_message>
<xml_diff>
--- a/04_Figures/S2/c_data/S2.xlsx
+++ b/04_Figures/S2/c_data/S2.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="218">
   <si>
     <t>sheet</t>
   </si>
@@ -170,12 +170,51 @@
     <t>Where the package came from.</t>
   </si>
   <si>
+    <t>modules</t>
+  </si>
+  <si>
+    <t>Acute_HRvLR</t>
+  </si>
+  <si>
+    <t>tan</t>
+  </si>
+  <si>
+    <t>red</t>
+  </si>
+  <si>
+    <t>greenyellow</t>
+  </si>
+  <si>
+    <t>Acute_change_HRvLR</t>
+  </si>
+  <si>
+    <t>blue</t>
+  </si>
+  <si>
+    <t>green</t>
+  </si>
+  <si>
+    <t>brown</t>
+  </si>
+  <si>
+    <t>Baseline_HRvLR</t>
+  </si>
+  <si>
+    <t>yellow</t>
+  </si>
+  <si>
+    <t>Trained_HRvLR</t>
+  </si>
+  <si>
+    <t>pink</t>
+  </si>
+  <si>
+    <t>Training_change_HRvLR</t>
+  </si>
+  <si>
     <t>proteins</t>
   </si>
   <si>
-    <t>Acute_HRvLR</t>
-  </si>
-  <si>
     <t>P33121</t>
   </si>
   <si>
@@ -194,7 +233,52 @@
     <t>NDRG2</t>
   </si>
   <si>
-    <t>Training_change_HRvLR</t>
+    <t>O94826</t>
+  </si>
+  <si>
+    <t>TOMM70</t>
+  </si>
+  <si>
+    <t>P17612</t>
+  </si>
+  <si>
+    <t>PRKACA</t>
+  </si>
+  <si>
+    <t>P51648</t>
+  </si>
+  <si>
+    <t>ALDH3A2</t>
+  </si>
+  <si>
+    <t>P34932</t>
+  </si>
+  <si>
+    <t>HSPA4</t>
+  </si>
+  <si>
+    <t>Q16890</t>
+  </si>
+  <si>
+    <t>TPD52L1</t>
+  </si>
+  <si>
+    <t>P22570</t>
+  </si>
+  <si>
+    <t>FDXR</t>
+  </si>
+  <si>
+    <t>Q9BYT8</t>
+  </si>
+  <si>
+    <t>NLN</t>
+  </si>
+  <si>
+    <t>P05413</t>
+  </si>
+  <si>
+    <t>FABP3</t>
   </si>
   <si>
     <t>P50395</t>
@@ -218,6 +302,90 @@
     <t>sets</t>
   </si>
   <si>
+    <t>GOBP|GOBP_COPII_COATED_VESICLE_BUDDING</t>
+  </si>
+  <si>
+    <t>GOBP</t>
+  </si>
+  <si>
+    <t>GOBP_COPII_COATED_VESICLE_BUDDING</t>
+  </si>
+  <si>
+    <t>GOBP|GOBP_VESICLE_BUDDING_FROM_MEMBRANE</t>
+  </si>
+  <si>
+    <t>GOBP_VESICLE_BUDDING_FROM_MEMBRANE</t>
+  </si>
+  <si>
+    <t>GOBP|GOBP_POSITIVE_REGULATION_OF_CELL_CYCLE_PROCESS</t>
+  </si>
+  <si>
+    <t>GOBP_POSITIVE_REGULATION_OF_CELL_CYCLE_PROCESS</t>
+  </si>
+  <si>
+    <t>KEGG_Legacy|KEGG_PPAR_SIGNALING_PATHWAY</t>
+  </si>
+  <si>
+    <t>KEGG_Legacy</t>
+  </si>
+  <si>
+    <t>KEGG_PPAR_SIGNALING_PATHWAY</t>
+  </si>
+  <si>
+    <t>Hallmark|HALLMARK_ADIPOGENESIS</t>
+  </si>
+  <si>
+    <t>Hallmark</t>
+  </si>
+  <si>
+    <t>HALLMARK_ADIPOGENESIS</t>
+  </si>
+  <si>
+    <t>GOBP|GOBP_REGULATION_OF_CALCIUM_ION_TRANSMEMBRANE_TRANSPORT</t>
+  </si>
+  <si>
+    <t>GOBP_REGULATION_OF_CALCIUM_ION_TRANSMEMBRANE_TRANSPORT</t>
+  </si>
+  <si>
+    <t>Hallmark|HALLMARK_IL2_STAT5_SIGNALING</t>
+  </si>
+  <si>
+    <t>HALLMARK_IL2_STAT5_SIGNALING</t>
+  </si>
+  <si>
+    <t>Reactome|REACTOME_GLYCEROPHOSPHOLIPID_BIOSYNTHESIS</t>
+  </si>
+  <si>
+    <t>Reactome</t>
+  </si>
+  <si>
+    <t>REACTOME_GLYCEROPHOSPHOLIPID_BIOSYNTHESIS</t>
+  </si>
+  <si>
+    <t>GOBP|GOBP_CYTOSKELETON_DEPENDENT_INTRACELLULAR_TRANSPORT</t>
+  </si>
+  <si>
+    <t>GOBP_CYTOSKELETON_DEPENDENT_INTRACELLULAR_TRANSPORT</t>
+  </si>
+  <si>
+    <t>Hallmark|HALLMARK_BILE_ACID_METABOLISM</t>
+  </si>
+  <si>
+    <t>HALLMARK_BILE_ACID_METABOLISM</t>
+  </si>
+  <si>
+    <t>GOBP|GOBP_RESPONSE_TO_ISCHEMIA</t>
+  </si>
+  <si>
+    <t>GOBP_RESPONSE_TO_ISCHEMIA</t>
+  </si>
+  <si>
+    <t>GOBP|GOBP_PROTEIN_TARGETING</t>
+  </si>
+  <si>
+    <t>GOBP_PROTEIN_TARGETING</t>
+  </si>
+  <si>
     <t>GO_Slim|TRANSMEMBRANE_TRANSPORT</t>
   </si>
   <si>
@@ -230,184 +398,16 @@
     <t>Reactome|REACTOME_FORMATION_OF_ATP_BY_CHEMIOSMOTIC_COUPLING</t>
   </si>
   <si>
-    <t>Reactome</t>
-  </si>
-  <si>
     <t>REACTOME_FORMATION_OF_ATP_BY_CHEMIOSMOTIC_COUPLING</t>
   </si>
   <si>
-    <t>Hallmark|HALLMARK_IL2_STAT5_SIGNALING</t>
-  </si>
-  <si>
-    <t>Hallmark</t>
-  </si>
-  <si>
-    <t>HALLMARK_IL2_STAT5_SIGNALING</t>
-  </si>
-  <si>
-    <t>Baseline_HRvLR</t>
-  </si>
-  <si>
-    <t>P34932</t>
-  </si>
-  <si>
-    <t>HSPA4</t>
-  </si>
-  <si>
-    <t>Q16890</t>
-  </si>
-  <si>
-    <t>TPD52L1</t>
-  </si>
-  <si>
-    <t>P22570</t>
-  </si>
-  <si>
-    <t>FDXR</t>
-  </si>
-  <si>
-    <t>Trained_HRvLR</t>
-  </si>
-  <si>
-    <t>O94826</t>
-  </si>
-  <si>
-    <t>TOMM70</t>
-  </si>
-  <si>
-    <t>Q9BYT8</t>
-  </si>
-  <si>
-    <t>NLN</t>
-  </si>
-  <si>
-    <t>P05413</t>
-  </si>
-  <si>
-    <t>FABP3</t>
-  </si>
-  <si>
-    <t>GOBP|GOBP_COPII_COATED_VESICLE_BUDDING</t>
-  </si>
-  <si>
-    <t>GOBP</t>
-  </si>
-  <si>
-    <t>GOBP_COPII_COATED_VESICLE_BUDDING</t>
-  </si>
-  <si>
-    <t>GOBP|GOBP_VESICLE_BUDDING_FROM_MEMBRANE</t>
-  </si>
-  <si>
-    <t>GOBP_VESICLE_BUDDING_FROM_MEMBRANE</t>
-  </si>
-  <si>
-    <t>GOBP|GOBP_POSITIVE_REGULATION_OF_CELL_CYCLE_PROCESS</t>
-  </si>
-  <si>
-    <t>GOBP_POSITIVE_REGULATION_OF_CELL_CYCLE_PROCESS</t>
-  </si>
-  <si>
-    <t>Acute_change_HRvLR</t>
-  </si>
-  <si>
-    <t>KEGG_Legacy|KEGG_PPAR_SIGNALING_PATHWAY</t>
-  </si>
-  <si>
-    <t>KEGG_Legacy</t>
-  </si>
-  <si>
-    <t>KEGG_PPAR_SIGNALING_PATHWAY</t>
-  </si>
-  <si>
-    <t>Hallmark|HALLMARK_ADIPOGENESIS</t>
-  </si>
-  <si>
-    <t>HALLMARK_ADIPOGENESIS</t>
-  </si>
-  <si>
-    <t>GOBP|GOBP_REGULATION_OF_CALCIUM_ION_TRANSMEMBRANE_TRANSPORT</t>
-  </si>
-  <si>
-    <t>GOBP_REGULATION_OF_CALCIUM_ION_TRANSMEMBRANE_TRANSPORT</t>
-  </si>
-  <si>
-    <t>P17612</t>
-  </si>
-  <si>
-    <t>PRKACA</t>
-  </si>
-  <si>
-    <t>P51648</t>
-  </si>
-  <si>
-    <t>ALDH3A2</t>
-  </si>
-  <si>
-    <t>Hallmark|HALLMARK_BILE_ACID_METABOLISM</t>
-  </si>
-  <si>
-    <t>HALLMARK_BILE_ACID_METABOLISM</t>
-  </si>
-  <si>
-    <t>GOBP|GOBP_RESPONSE_TO_ISCHEMIA</t>
-  </si>
-  <si>
-    <t>GOBP_RESPONSE_TO_ISCHEMIA</t>
-  </si>
-  <si>
-    <t>GOBP|GOBP_PROTEIN_TARGETING</t>
-  </si>
-  <si>
-    <t>GOBP_PROTEIN_TARGETING</t>
-  </si>
-  <si>
-    <t>Reactome|REACTOME_GLYCEROPHOSPHOLIPID_BIOSYNTHESIS</t>
-  </si>
-  <si>
-    <t>REACTOME_GLYCEROPHOSPHOLIPID_BIOSYNTHESIS</t>
-  </si>
-  <si>
-    <t>GOBP|GOBP_CYTOSKELETON_DEPENDENT_INTRACELLULAR_TRANSPORT</t>
-  </si>
-  <si>
-    <t>GOBP_CYTOSKELETON_DEPENDENT_INTRACELLULAR_TRANSPORT</t>
-  </si>
-  <si>
-    <t>modules</t>
-  </si>
-  <si>
-    <t>blue</t>
-  </si>
-  <si>
-    <t>green</t>
-  </si>
-  <si>
-    <t>brown</t>
-  </si>
-  <si>
-    <t>tan</t>
-  </si>
-  <si>
-    <t>red</t>
-  </si>
-  <si>
-    <t>greenyellow</t>
-  </si>
-  <si>
-    <t>pink</t>
-  </si>
-  <si>
-    <t>yellow</t>
-  </si>
-  <si>
     <t>classification</t>
   </si>
   <si>
     <t>02_HRvLR/06_Classification/c_data/classification.rds</t>
   </si>
   <si>
-    <t>bcbee59ce70db2c2438a80802c34a45e</t>
+    <t>c97416b8a9f513603e16f34826cd10f2</t>
   </si>
   <si>
     <t>characterisation</t>
@@ -488,12 +488,27 @@
     <t>4.0.3</t>
   </si>
   <si>
+    <t>ggtext</t>
+  </si>
+  <si>
+    <t>0.2.0</t>
+  </si>
+  <si>
+    <t>CRAN (R 4.6.1)</t>
+  </si>
+  <si>
     <t>glue</t>
   </si>
   <si>
     <t>1.8.1</t>
   </si>
   <si>
+    <t>gridtext</t>
+  </si>
+  <si>
+    <t>0.1.6</t>
+  </si>
+  <si>
     <t>gtable</t>
   </si>
   <si>
@@ -548,6 +563,12 @@
     <t>1.1-3</t>
   </si>
   <si>
+    <t>Rcpp</t>
+  </si>
+  <si>
+    <t>1.1.1-1.1</t>
+  </si>
+  <si>
     <t>readr</t>
   </si>
   <si>
@@ -572,9 +593,6 @@
     <t>1.3.0</t>
   </si>
   <si>
-    <t>CRAN (R 4.6.1)</t>
-  </si>
-  <si>
     <t>rprojroot</t>
   </si>
   <si>
@@ -642,6 +660,12 @@
   </si>
   <si>
     <t>3.0.2</t>
+  </si>
+  <si>
+    <t>xml2</t>
+  </si>
+  <si>
+    <t>1.5.2</t>
   </si>
   <si>
     <t>yaml</t>
@@ -1328,22 +1352,28 @@
         <v>52</v>
       </c>
       <c r="F2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G2">
+        <v>0.21875</v>
+      </c>
+      <c r="H2">
         <v>0</v>
       </c>
+      <c r="I2">
+        <v>0.48269945453518</v>
+      </c>
       <c r="J2">
-        <v>0.0001554001554001554</v>
+        <v>0.06495726495726495</v>
       </c>
       <c r="K2">
-        <v>0.31996891996892</v>
+        <v>0.6096969696969696</v>
       </c>
       <c r="L2">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>2059</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1357,31 +1387,31 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G3">
-        <v>0.03125</v>
+        <v>0.25</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>0.1044564071121033</v>
+        <v>0.503594433115469</v>
       </c>
       <c r="J3">
-        <v>0.0006216006216006216</v>
+        <v>0.1048951048951049</v>
       </c>
       <c r="K3">
-        <v>0.6399378399378399</v>
+        <v>0.6096969696969696</v>
       </c>
       <c r="L3">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="M3">
-        <v>2059</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1395,31 +1425,31 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="G4">
-        <v>0.953125</v>
+        <v>0.28125</v>
       </c>
       <c r="H4">
-        <v>0.8508978158344715</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>0.568532686305406</v>
       </c>
       <c r="J4">
-        <v>0.001087801087801088</v>
+        <v>0.1605283605283605</v>
       </c>
       <c r="K4">
-        <v>0.6754899421566088</v>
+        <v>0.6096969696969696</v>
       </c>
       <c r="L4">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="M4">
-        <v>2059</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1427,37 +1457,37 @@
         <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G5">
-        <v>0.03125</v>
+        <v>0.796875</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>0.5524269785900641</v>
       </c>
       <c r="I5">
-        <v>0.1044564071121033</v>
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>0.0006216006216006216</v>
+        <v>0.04988344988344988</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>0.4545454545454545</v>
       </c>
       <c r="L5">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>2059</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1465,37 +1495,37 @@
         <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C6">
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="G6">
-        <v>0.0625</v>
+        <v>0.765625</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>0.5211769785900641</v>
       </c>
       <c r="I6">
-        <v>0.1759108782323425</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>0.001709401709401709</v>
+        <v>0.08298368298368297</v>
       </c>
       <c r="K6">
-        <v>1</v>
+        <v>0.4545454545454545</v>
       </c>
       <c r="L6">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="M6">
-        <v>2059</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1503,160 +1533,151 @@
         <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C7">
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="F7" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G7">
-        <v>0.078125</v>
+        <v>0.25</v>
       </c>
       <c r="H7">
         <v>0</v>
       </c>
       <c r="I7">
-        <v>0.2080534835327822</v>
+        <v>0.5119112043058992</v>
       </c>
       <c r="J7">
-        <v>0.002952602952602953</v>
+        <v>0.1048951048951049</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>0.4545454545454545</v>
       </c>
       <c r="L7">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="M7">
-        <v>2059</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>66</v>
-      </c>
-      <c r="E8" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="F8" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="G8">
-        <v>0.96875</v>
+        <v>0.3125</v>
       </c>
       <c r="H8">
-        <v>0.8955435928878968</v>
+        <v>0.03470121704984507</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0.5902987829501549</v>
       </c>
       <c r="J8">
-        <v>0.0006216006216006216</v>
+        <v>0.2344988344988345</v>
       </c>
       <c r="K8">
-        <v>0.03605283605283605</v>
+        <v>1</v>
       </c>
       <c r="L8">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="M8">
-        <v>1422</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C9">
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>69</v>
-      </c>
-      <c r="E9" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="G9">
-        <v>0.90625</v>
+        <v>0.671875</v>
       </c>
       <c r="H9">
-        <v>0.7181793348793176</v>
+        <v>0.3722648663130612</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0.9714851336869388</v>
       </c>
       <c r="J9">
-        <v>0.004506604506604228</v>
+        <v>0.2786324786324786</v>
       </c>
       <c r="K9">
-        <v>0.9963775167658665</v>
+        <v>1</v>
       </c>
       <c r="L9">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="M9">
-        <v>1422</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C10">
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>72</v>
-      </c>
-      <c r="E10" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="F10" t="s">
-        <v>74</v>
+        <v>52</v>
       </c>
       <c r="G10">
-        <v>0.109375</v>
+        <v>0.390625</v>
       </c>
       <c r="H10">
+        <v>0.08745853842350808</v>
+      </c>
+      <c r="I10">
+        <v>0.693791461576492</v>
+      </c>
+      <c r="J10">
+        <v>0.5053613053613053</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10">
         <v>0</v>
       </c>
-      <c r="I10">
-        <v>0.2689246653106777</v>
-      </c>
-      <c r="J10">
-        <v>0.006993006993006993</v>
-      </c>
-      <c r="K10">
-        <v>0.2447552447552448</v>
-      </c>
-      <c r="L10">
-        <v>30</v>
-      </c>
       <c r="M10">
-        <v>1422</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1664,37 +1685,37 @@
         <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="F11" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="G11">
-        <v>0.046875</v>
+        <v>0.234375</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>0.1491021841655284</v>
+        <v>0.4957741584509279</v>
       </c>
       <c r="J11">
-        <v>0.001087801087801088</v>
+        <v>0.08298368298368297</v>
       </c>
       <c r="K11">
-        <v>1</v>
+        <v>0.5393939393939393</v>
       </c>
       <c r="L11">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="M11">
-        <v>2059</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -1702,37 +1723,37 @@
         <v>50</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="C12">
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="F12" t="s">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="G12">
-        <v>0.921875</v>
+        <v>0.234375</v>
       </c>
       <c r="H12">
-        <v>0.7919465164672178</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>0.4788230214099359</v>
       </c>
       <c r="J12">
-        <v>0.002952602952602801</v>
+        <v>0.08298368298368297</v>
       </c>
       <c r="K12">
-        <v>1</v>
+        <v>0.5393939393939393</v>
       </c>
       <c r="L12">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="M12">
-        <v>2059</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -1740,37 +1761,37 @@
         <v>50</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="C13">
         <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="F13" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="G13">
-        <v>0.109375</v>
+        <v>0.3125</v>
       </c>
       <c r="H13">
+        <v>0.03470121704984507</v>
+      </c>
+      <c r="I13">
+        <v>0.5902987829501549</v>
+      </c>
+      <c r="J13">
+        <v>0.2344988344988345</v>
+      </c>
+      <c r="K13">
+        <v>0.8389898989898988</v>
+      </c>
+      <c r="L13">
         <v>0</v>
       </c>
-      <c r="I13">
-        <v>0.2787019102242969</v>
-      </c>
-      <c r="J13">
-        <v>0.006216006216006216</v>
-      </c>
-      <c r="K13">
-        <v>1</v>
-      </c>
-      <c r="L13">
-        <v>56</v>
-      </c>
       <c r="M13">
-        <v>2059</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -1778,37 +1799,37 @@
         <v>50</v>
       </c>
       <c r="B14" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>83</v>
+        <v>53</v>
       </c>
       <c r="F14" t="s">
-        <v>84</v>
+        <v>53</v>
       </c>
       <c r="G14">
-        <v>0.046875</v>
+        <v>0.734375</v>
       </c>
       <c r="H14">
+        <v>0.4570589259861157</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>0.1303807303807304</v>
+      </c>
+      <c r="K14">
+        <v>0.8444444444444442</v>
+      </c>
+      <c r="L14">
         <v>0</v>
       </c>
-      <c r="I14">
-        <v>0.1491021841655284</v>
-      </c>
-      <c r="J14">
-        <v>0.001087801087801088</v>
-      </c>
-      <c r="K14">
-        <v>0.9435925551057128</v>
-      </c>
-      <c r="L14">
-        <v>103</v>
-      </c>
       <c r="M14">
-        <v>2059</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -1816,37 +1837,37 @@
         <v>50</v>
       </c>
       <c r="B15" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="C15">
         <v>2</v>
       </c>
       <c r="D15" t="s">
-        <v>85</v>
+        <v>56</v>
       </c>
       <c r="F15" t="s">
-        <v>86</v>
+        <v>56</v>
       </c>
       <c r="G15">
-        <v>0.9375</v>
+        <v>0.28125</v>
       </c>
       <c r="H15">
-        <v>0.8150022509662467</v>
+        <v>0.009300267543375791</v>
       </c>
       <c r="I15">
-        <v>1</v>
+        <v>0.5531997324566242</v>
       </c>
       <c r="J15">
-        <v>0.001398601398602262</v>
+        <v>0.1605283605283605</v>
       </c>
       <c r="K15">
-        <v>0.9435925551057128</v>
+        <v>0.8444444444444442</v>
       </c>
       <c r="L15">
-        <v>103</v>
+        <v>0</v>
       </c>
       <c r="M15">
-        <v>2059</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -1854,42 +1875,42 @@
         <v>50</v>
       </c>
       <c r="B16" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="C16">
         <v>3</v>
       </c>
       <c r="D16" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="F16" t="s">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="G16">
-        <v>0.0625</v>
+        <v>0.296875</v>
       </c>
       <c r="H16">
+        <v>0.02739983885770896</v>
+      </c>
+      <c r="I16">
+        <v>0.5663501611422911</v>
+      </c>
+      <c r="J16">
+        <v>0.1948717948717948</v>
+      </c>
+      <c r="K16">
+        <v>0.8444444444444442</v>
+      </c>
+      <c r="L16">
         <v>0</v>
       </c>
-      <c r="I16">
-        <v>0.1759108782323425</v>
-      </c>
-      <c r="J16">
-        <v>0.001864801864801865</v>
-      </c>
-      <c r="K16">
-        <v>0.9435925551057128</v>
-      </c>
-      <c r="L16">
-        <v>103</v>
-      </c>
       <c r="M16">
-        <v>2059</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:13">
       <c r="A17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B17" t="s">
         <v>51</v>
@@ -1898,39 +1919,30 @@
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>89</v>
-      </c>
-      <c r="E17" t="s">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="F17" t="s">
-        <v>91</v>
+        <v>66</v>
       </c>
       <c r="G17">
-        <v>0.953125</v>
-      </c>
-      <c r="H17">
-        <v>0.8619837581524826</v>
-      </c>
-      <c r="I17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17">
-        <v>0.001087801087801088</v>
+        <v>0.0001554001554001554</v>
       </c>
       <c r="K17">
-        <v>0.5183372183372184</v>
+        <v>0.31996891996892</v>
       </c>
       <c r="L17">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="M17">
-        <v>1422</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="18" spans="1:13">
       <c r="A18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B18" t="s">
         <v>51</v>
@@ -1939,39 +1951,36 @@
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>92</v>
-      </c>
-      <c r="E18" t="s">
-        <v>90</v>
+        <v>67</v>
       </c>
       <c r="F18" t="s">
-        <v>93</v>
+        <v>68</v>
       </c>
       <c r="G18">
-        <v>0.953125</v>
+        <v>0.03125</v>
       </c>
       <c r="H18">
-        <v>0.8619837581524826</v>
+        <v>0</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>0.1044564071121033</v>
       </c>
       <c r="J18">
-        <v>0.001087801087801088</v>
+        <v>0.0006216006216006216</v>
       </c>
       <c r="K18">
-        <v>0.5183372183372184</v>
+        <v>0.6399378399378399</v>
       </c>
       <c r="L18">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="M18">
-        <v>1422</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="19" spans="1:13">
       <c r="A19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B19" t="s">
         <v>51</v>
@@ -1980,192 +1989,180 @@
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>94</v>
-      </c>
-      <c r="E19" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="F19" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="G19">
-        <v>0.9375</v>
+        <v>0.953125</v>
       </c>
       <c r="H19">
-        <v>0.8065443978470503</v>
+        <v>0.8508978158344715</v>
       </c>
       <c r="I19">
         <v>1</v>
       </c>
       <c r="J19">
-        <v>0.001864801864801865</v>
+        <v>0.001087801087801088</v>
       </c>
       <c r="K19">
-        <v>0.5553613053613053</v>
+        <v>0.6754899421566088</v>
       </c>
       <c r="L19">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="M19">
-        <v>1422</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="20" spans="1:13">
       <c r="A20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B20" t="s">
-        <v>96</v>
+        <v>55</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>97</v>
-      </c>
-      <c r="E20" t="s">
-        <v>98</v>
+        <v>71</v>
       </c>
       <c r="F20" t="s">
-        <v>99</v>
+        <v>72</v>
       </c>
       <c r="G20">
-        <v>0.046875</v>
+        <v>0.9375</v>
       </c>
       <c r="H20">
-        <v>0</v>
+        <v>0.8240891217676575</v>
       </c>
       <c r="I20">
-        <v>0.1380162418475174</v>
+        <v>1</v>
       </c>
       <c r="J20">
-        <v>0.001087801087801088</v>
+        <v>0.001864801864801865</v>
       </c>
       <c r="K20">
-        <v>0.05982905982905983</v>
+        <v>0.7933475960873221</v>
       </c>
       <c r="L20">
-        <v>73</v>
+        <v>127</v>
       </c>
       <c r="M20">
-        <v>1422</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="21" spans="1:13">
       <c r="A21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>96</v>
+        <v>55</v>
       </c>
       <c r="C21">
         <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>100</v>
-      </c>
-      <c r="E21" t="s">
         <v>73</v>
       </c>
       <c r="F21" t="s">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="G21">
-        <v>0.078125</v>
+        <v>0.9375</v>
       </c>
       <c r="H21">
-        <v>0</v>
+        <v>0.8240891217676575</v>
       </c>
       <c r="I21">
-        <v>0.2080534835327822</v>
+        <v>1</v>
       </c>
       <c r="J21">
-        <v>0.002952602952602953</v>
+        <v>0.001864801864801865</v>
       </c>
       <c r="K21">
-        <v>0.1033411033411033</v>
+        <v>0.7933475960873221</v>
       </c>
       <c r="L21">
-        <v>73</v>
+        <v>127</v>
       </c>
       <c r="M21">
-        <v>1422</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="22" spans="1:13">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B22" t="s">
-        <v>96</v>
+        <v>55</v>
       </c>
       <c r="C22">
         <v>3</v>
       </c>
       <c r="D22" t="s">
-        <v>102</v>
-      </c>
-      <c r="E22" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="F22" t="s">
-        <v>103</v>
+        <v>76</v>
       </c>
       <c r="G22">
-        <v>0.09375</v>
+        <v>0.9375</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>0.8240891217676575</v>
       </c>
       <c r="I22">
-        <v>0.2437784898861034</v>
+        <v>1</v>
       </c>
       <c r="J22">
-        <v>0.004662004662004662</v>
+        <v>0.001864801864801865</v>
       </c>
       <c r="K22">
-        <v>0.7622873377474604</v>
+        <v>0.7933475960873221</v>
       </c>
       <c r="L22">
-        <v>73</v>
+        <v>127</v>
       </c>
       <c r="M22">
-        <v>1422</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="23" spans="1:13">
       <c r="A23" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="B23" t="s">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="F23" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="G23">
-        <v>0.9375</v>
+        <v>0.046875</v>
       </c>
       <c r="H23">
-        <v>0.8240891217676575</v>
+        <v>0</v>
       </c>
       <c r="I23">
-        <v>1</v>
+        <v>0.1491021841655284</v>
       </c>
       <c r="J23">
-        <v>0.001864801864801865</v>
+        <v>0.001087801087801088</v>
       </c>
       <c r="K23">
-        <v>0.7933475960873221</v>
+        <v>1</v>
       </c>
       <c r="L23">
-        <v>127</v>
+        <v>56</v>
       </c>
       <c r="M23">
         <v>2059</v>
@@ -2173,37 +2170,37 @@
     </row>
     <row r="24" spans="1:13">
       <c r="A24" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="B24" t="s">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="C24">
         <v>2</v>
       </c>
       <c r="D24" t="s">
-        <v>104</v>
+        <v>79</v>
       </c>
       <c r="F24" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="G24">
-        <v>0.9375</v>
+        <v>0.921875</v>
       </c>
       <c r="H24">
-        <v>0.8240891217676575</v>
+        <v>0.7919465164672178</v>
       </c>
       <c r="I24">
         <v>1</v>
       </c>
       <c r="J24">
-        <v>0.001864801864801865</v>
+        <v>0.002952602952602801</v>
       </c>
       <c r="K24">
-        <v>0.7933475960873221</v>
+        <v>1</v>
       </c>
       <c r="L24">
-        <v>127</v>
+        <v>56</v>
       </c>
       <c r="M24">
         <v>2059</v>
@@ -2211,37 +2208,37 @@
     </row>
     <row r="25" spans="1:13">
       <c r="A25" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="B25" t="s">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="C25">
         <v>3</v>
       </c>
       <c r="D25" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="F25" t="s">
-        <v>107</v>
+        <v>82</v>
       </c>
       <c r="G25">
-        <v>0.9375</v>
+        <v>0.109375</v>
       </c>
       <c r="H25">
-        <v>0.8240891217676575</v>
+        <v>0</v>
       </c>
       <c r="I25">
-        <v>1</v>
+        <v>0.2787019102242969</v>
       </c>
       <c r="J25">
-        <v>0.001864801864801865</v>
+        <v>0.006216006216006216</v>
       </c>
       <c r="K25">
-        <v>0.7933475960873221</v>
+        <v>1</v>
       </c>
       <c r="L25">
-        <v>127</v>
+        <v>56</v>
       </c>
       <c r="M25">
         <v>2059</v>
@@ -2249,674 +2246,689 @@
     </row>
     <row r="26" spans="1:13">
       <c r="A26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B26" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="C26">
         <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>108</v>
-      </c>
-      <c r="E26" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F26" t="s">
-        <v>109</v>
+        <v>72</v>
       </c>
       <c r="G26">
-        <v>0.078125</v>
+        <v>0.046875</v>
       </c>
       <c r="H26">
         <v>0</v>
       </c>
       <c r="I26">
-        <v>0.2160564396721562</v>
+        <v>0.1491021841655284</v>
       </c>
       <c r="J26">
-        <v>0.002952602952602953</v>
+        <v>0.001087801087801088</v>
       </c>
       <c r="K26">
-        <v>0.1033411033411033</v>
+        <v>0.9435925551057128</v>
       </c>
       <c r="L26">
-        <v>18</v>
+        <v>103</v>
       </c>
       <c r="M26">
-        <v>1422</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="27" spans="1:13">
       <c r="A27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B27" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="C27">
         <v>2</v>
       </c>
       <c r="D27" t="s">
-        <v>110</v>
-      </c>
-      <c r="E27" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="F27" t="s">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="G27">
-        <v>0.921875</v>
+        <v>0.9375</v>
       </c>
       <c r="H27">
-        <v>0.7919465164672178</v>
+        <v>0.8150022509662467</v>
       </c>
       <c r="I27">
         <v>1</v>
       </c>
       <c r="J27">
-        <v>0.002952602952602953</v>
+        <v>0.001398601398602262</v>
       </c>
       <c r="K27">
-        <v>1</v>
+        <v>0.9435925551057128</v>
       </c>
       <c r="L27">
-        <v>18</v>
+        <v>103</v>
       </c>
       <c r="M27">
-        <v>1422</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="28" spans="1:13">
       <c r="A28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B28" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="C28">
         <v>3</v>
       </c>
       <c r="D28" t="s">
-        <v>112</v>
-      </c>
-      <c r="E28" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F28" t="s">
-        <v>113</v>
+        <v>86</v>
       </c>
       <c r="G28">
-        <v>0.140625</v>
+        <v>0.0625</v>
       </c>
       <c r="H28">
         <v>0</v>
       </c>
       <c r="I28">
-        <v>0.3417761725521024</v>
+        <v>0.1759108782323425</v>
       </c>
       <c r="J28">
-        <v>0.01476301476301476</v>
+        <v>0.001864801864801865</v>
       </c>
       <c r="K28">
-        <v>1</v>
+        <v>0.9435925551057128</v>
       </c>
       <c r="L28">
-        <v>18</v>
+        <v>103</v>
       </c>
       <c r="M28">
-        <v>1422</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="29" spans="1:13">
       <c r="A29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>72</v>
-      </c>
-      <c r="E29" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="F29" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="G29">
-        <v>0.890625</v>
+        <v>0.03125</v>
       </c>
       <c r="H29">
-        <v>0.7181621398400233</v>
+        <v>0</v>
       </c>
       <c r="I29">
-        <v>1</v>
+        <v>0.1044564071121033</v>
       </c>
       <c r="J29">
-        <v>0.006993006993006993</v>
+        <v>0.0006216006216006216</v>
       </c>
       <c r="K29">
-        <v>0.2447552447552448</v>
+        <v>1</v>
       </c>
       <c r="L29">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="M29">
-        <v>1422</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="30" spans="1:13">
       <c r="A30" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B30" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>114</v>
-      </c>
-      <c r="E30" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="F30" t="s">
-        <v>115</v>
+        <v>90</v>
       </c>
       <c r="G30">
-        <v>0.109375</v>
+        <v>0.0625</v>
       </c>
       <c r="H30">
         <v>0</v>
       </c>
       <c r="I30">
-        <v>0.3259224725546371</v>
+        <v>0.1759108782323425</v>
       </c>
       <c r="J30">
-        <v>0.006993006993006993</v>
+        <v>0.001709401709401709</v>
       </c>
       <c r="K30">
-        <v>0.9934153701595559</v>
+        <v>1</v>
       </c>
       <c r="L30">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="M30">
-        <v>1422</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="31" spans="1:13">
       <c r="A31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B31" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C31">
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>116</v>
-      </c>
-      <c r="E31" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F31" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="G31">
-        <v>0.890625</v>
+        <v>0.078125</v>
       </c>
       <c r="H31">
-        <v>0.7310753346893223</v>
+        <v>0</v>
       </c>
       <c r="I31">
-        <v>1</v>
+        <v>0.2080534835327822</v>
       </c>
       <c r="J31">
-        <v>0.006993006993006993</v>
+        <v>0.002952602952602953</v>
       </c>
       <c r="K31">
         <v>1</v>
       </c>
       <c r="L31">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="M31">
-        <v>1422</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="32" spans="1:13">
       <c r="A32" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B32" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32" t="s">
+        <v>94</v>
+      </c>
+      <c r="E32" t="s">
+        <v>95</v>
+      </c>
+      <c r="F32" t="s">
         <v>96</v>
       </c>
-      <c r="C32">
-        <v>1</v>
-      </c>
-      <c r="D32" t="s">
-        <v>119</v>
-      </c>
-      <c r="F32" t="s">
-        <v>119</v>
-      </c>
       <c r="G32">
-        <v>0.796875</v>
+        <v>0.953125</v>
       </c>
       <c r="H32">
-        <v>0.5524269785900641</v>
+        <v>0.8619837581524826</v>
       </c>
       <c r="I32">
         <v>1</v>
       </c>
       <c r="J32">
-        <v>0.04988344988344988</v>
+        <v>0.001087801087801088</v>
       </c>
       <c r="K32">
-        <v>0.4545454545454545</v>
+        <v>0.5183372183372184</v>
       </c>
       <c r="L32">
-        <v>1</v>
+        <v>121</v>
       </c>
       <c r="M32">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="33" spans="1:13">
       <c r="A33" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B33" t="s">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="C33">
         <v>2</v>
       </c>
       <c r="D33" t="s">
-        <v>120</v>
+        <v>97</v>
+      </c>
+      <c r="E33" t="s">
+        <v>95</v>
       </c>
       <c r="F33" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="G33">
-        <v>0.765625</v>
+        <v>0.953125</v>
       </c>
       <c r="H33">
-        <v>0.5211769785900641</v>
+        <v>0.8619837581524826</v>
       </c>
       <c r="I33">
         <v>1</v>
       </c>
       <c r="J33">
-        <v>0.08298368298368297</v>
+        <v>0.001087801087801088</v>
       </c>
       <c r="K33">
-        <v>0.4545454545454545</v>
+        <v>0.5183372183372184</v>
       </c>
       <c r="L33">
-        <v>1</v>
+        <v>121</v>
       </c>
       <c r="M33">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="34" spans="1:13">
       <c r="A34" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B34" t="s">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="C34">
         <v>3</v>
       </c>
       <c r="D34" t="s">
+        <v>99</v>
+      </c>
+      <c r="E34" t="s">
+        <v>95</v>
+      </c>
+      <c r="F34" t="s">
+        <v>100</v>
+      </c>
+      <c r="G34">
+        <v>0.9375</v>
+      </c>
+      <c r="H34">
+        <v>0.8065443978470503</v>
+      </c>
+      <c r="I34">
+        <v>1</v>
+      </c>
+      <c r="J34">
+        <v>0.001864801864801865</v>
+      </c>
+      <c r="K34">
+        <v>0.5553613053613053</v>
+      </c>
+      <c r="L34">
         <v>121</v>
       </c>
-      <c r="F34" t="s">
-        <v>121</v>
-      </c>
-      <c r="G34">
-        <v>0.25</v>
-      </c>
-      <c r="H34">
-        <v>0</v>
-      </c>
-      <c r="I34">
-        <v>0.5119112043058992</v>
-      </c>
-      <c r="J34">
-        <v>0.1048951048951049</v>
-      </c>
-      <c r="K34">
-        <v>0.4545454545454545</v>
-      </c>
-      <c r="L34">
-        <v>1</v>
-      </c>
       <c r="M34">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="35" spans="1:13">
       <c r="A35" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B35" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C35">
         <v>1</v>
       </c>
       <c r="D35" t="s">
-        <v>122</v>
+        <v>101</v>
+      </c>
+      <c r="E35" t="s">
+        <v>102</v>
       </c>
       <c r="F35" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="G35">
-        <v>0.21875</v>
+        <v>0.046875</v>
       </c>
       <c r="H35">
         <v>0</v>
       </c>
       <c r="I35">
-        <v>0.48269945453518</v>
+        <v>0.1380162418475174</v>
       </c>
       <c r="J35">
-        <v>0.06495726495726495</v>
+        <v>0.001087801087801088</v>
       </c>
       <c r="K35">
-        <v>0.6096969696969696</v>
+        <v>0.05982905982905983</v>
       </c>
       <c r="L35">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="M35">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="36" spans="1:13">
       <c r="A36" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B36" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C36">
         <v>2</v>
       </c>
       <c r="D36" t="s">
-        <v>123</v>
+        <v>104</v>
+      </c>
+      <c r="E36" t="s">
+        <v>105</v>
       </c>
       <c r="F36" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="G36">
-        <v>0.25</v>
+        <v>0.078125</v>
       </c>
       <c r="H36">
         <v>0</v>
       </c>
       <c r="I36">
-        <v>0.503594433115469</v>
+        <v>0.2080534835327822</v>
       </c>
       <c r="J36">
-        <v>0.1048951048951049</v>
+        <v>0.002952602952602953</v>
       </c>
       <c r="K36">
-        <v>0.6096969696969696</v>
+        <v>0.1033411033411033</v>
       </c>
       <c r="L36">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="M36">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="37" spans="1:13">
       <c r="A37" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B37" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C37">
         <v>3</v>
       </c>
       <c r="D37" t="s">
-        <v>124</v>
+        <v>107</v>
+      </c>
+      <c r="E37" t="s">
+        <v>95</v>
       </c>
       <c r="F37" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="G37">
-        <v>0.28125</v>
+        <v>0.09375</v>
       </c>
       <c r="H37">
         <v>0</v>
       </c>
       <c r="I37">
-        <v>0.568532686305406</v>
+        <v>0.2437784898861034</v>
       </c>
       <c r="J37">
-        <v>0.1605283605283605</v>
+        <v>0.004662004662004662</v>
       </c>
       <c r="K37">
-        <v>0.6096969696969696</v>
+        <v>0.7622873377474604</v>
       </c>
       <c r="L37">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="M37">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="38" spans="1:13">
       <c r="A38" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B38" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="C38">
         <v>1</v>
       </c>
       <c r="D38" t="s">
-        <v>119</v>
+        <v>109</v>
+      </c>
+      <c r="E38" t="s">
+        <v>105</v>
       </c>
       <c r="F38" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="G38">
-        <v>0.234375</v>
+        <v>0.890625</v>
       </c>
       <c r="H38">
-        <v>0</v>
+        <v>0.7181621398400233</v>
       </c>
       <c r="I38">
-        <v>0.4957741584509279</v>
+        <v>1</v>
       </c>
       <c r="J38">
-        <v>0.08298368298368297</v>
+        <v>0.006993006993006993</v>
       </c>
       <c r="K38">
-        <v>0.5393939393939393</v>
+        <v>0.2447552447552448</v>
       </c>
       <c r="L38">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="M38">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="39" spans="1:13">
       <c r="A39" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B39" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="C39">
         <v>2</v>
       </c>
       <c r="D39" t="s">
-        <v>120</v>
+        <v>111</v>
+      </c>
+      <c r="E39" t="s">
+        <v>112</v>
       </c>
       <c r="F39" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="G39">
-        <v>0.234375</v>
+        <v>0.109375</v>
       </c>
       <c r="H39">
         <v>0</v>
       </c>
       <c r="I39">
-        <v>0.4788230214099359</v>
+        <v>0.3259224725546371</v>
       </c>
       <c r="J39">
-        <v>0.08298368298368297</v>
+        <v>0.006993006993006993</v>
       </c>
       <c r="K39">
-        <v>0.5393939393939393</v>
+        <v>0.9934153701595559</v>
       </c>
       <c r="L39">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="M39">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="40" spans="1:13">
       <c r="A40" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B40" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="C40">
         <v>3</v>
       </c>
       <c r="D40" t="s">
-        <v>125</v>
+        <v>114</v>
+      </c>
+      <c r="E40" t="s">
+        <v>95</v>
       </c>
       <c r="F40" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="G40">
-        <v>0.3125</v>
+        <v>0.890625</v>
       </c>
       <c r="H40">
-        <v>0.03470121704984507</v>
+        <v>0.7310753346893223</v>
       </c>
       <c r="I40">
-        <v>0.5902987829501549</v>
+        <v>1</v>
       </c>
       <c r="J40">
-        <v>0.2344988344988345</v>
+        <v>0.006993006993006993</v>
       </c>
       <c r="K40">
-        <v>0.8389898989898988</v>
+        <v>1</v>
       </c>
       <c r="L40">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="M40">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="41" spans="1:13">
       <c r="A41" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B41" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>123</v>
+        <v>116</v>
+      </c>
+      <c r="E41" t="s">
+        <v>105</v>
       </c>
       <c r="F41" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="G41">
-        <v>0.734375</v>
+        <v>0.078125</v>
       </c>
       <c r="H41">
-        <v>0.4570589259861157</v>
+        <v>0</v>
       </c>
       <c r="I41">
-        <v>1</v>
+        <v>0.2160564396721562</v>
       </c>
       <c r="J41">
-        <v>0.1303807303807304</v>
+        <v>0.002952602952602953</v>
       </c>
       <c r="K41">
-        <v>0.8444444444444442</v>
+        <v>0.1033411033411033</v>
       </c>
       <c r="L41">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="M41">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="42" spans="1:13">
       <c r="A42" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B42" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C42">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>119</v>
+        <v>118</v>
+      </c>
+      <c r="E42" t="s">
+        <v>95</v>
       </c>
       <c r="F42" t="s">
         <v>119</v>
       </c>
       <c r="G42">
-        <v>0.28125</v>
+        <v>0.921875</v>
       </c>
       <c r="H42">
-        <v>0.009300267543375791</v>
+        <v>0.7919465164672178</v>
       </c>
       <c r="I42">
-        <v>0.5531997324566242</v>
+        <v>1</v>
       </c>
       <c r="J42">
-        <v>0.1605283605283605</v>
+        <v>0.002952602952602953</v>
       </c>
       <c r="K42">
-        <v>0.8444444444444442</v>
+        <v>1</v>
       </c>
       <c r="L42">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="M42">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="43" spans="1:13">
       <c r="A43" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B43" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C43">
         <v>3</v>
@@ -2924,143 +2936,155 @@
       <c r="D43" t="s">
         <v>120</v>
       </c>
+      <c r="E43" t="s">
+        <v>95</v>
+      </c>
       <c r="F43" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G43">
-        <v>0.296875</v>
+        <v>0.140625</v>
       </c>
       <c r="H43">
-        <v>0.02739983885770896</v>
+        <v>0</v>
       </c>
       <c r="I43">
-        <v>0.5663501611422911</v>
+        <v>0.3417761725521024</v>
       </c>
       <c r="J43">
-        <v>0.1948717948717948</v>
+        <v>0.01476301476301476</v>
       </c>
       <c r="K43">
-        <v>0.8444444444444442</v>
+        <v>1</v>
       </c>
       <c r="L43">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="M43">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="44" spans="1:13">
       <c r="A44" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B44" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C44">
         <v>1</v>
       </c>
       <c r="D44" t="s">
+        <v>122</v>
+      </c>
+      <c r="E44" t="s">
         <v>123</v>
       </c>
       <c r="F44" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G44">
-        <v>0.3125</v>
+        <v>0.96875</v>
       </c>
       <c r="H44">
-        <v>0.03470121704984507</v>
+        <v>0.8955435928878968</v>
       </c>
       <c r="I44">
-        <v>0.5902987829501549</v>
+        <v>1</v>
       </c>
       <c r="J44">
-        <v>0.2344988344988345</v>
+        <v>0.0006216006216006216</v>
       </c>
       <c r="K44">
-        <v>1</v>
+        <v>0.03605283605283605</v>
       </c>
       <c r="L44">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="M44">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="45" spans="1:13">
       <c r="A45" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B45" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C45">
         <v>2</v>
       </c>
       <c r="D45" t="s">
-        <v>126</v>
+        <v>125</v>
+      </c>
+      <c r="E45" t="s">
+        <v>112</v>
       </c>
       <c r="F45" t="s">
         <v>126</v>
       </c>
       <c r="G45">
-        <v>0.671875</v>
+        <v>0.90625</v>
       </c>
       <c r="H45">
-        <v>0.3722648663130612</v>
+        <v>0.7181793348793176</v>
       </c>
       <c r="I45">
-        <v>0.9714851336869388</v>
+        <v>1</v>
       </c>
       <c r="J45">
-        <v>0.2786324786324786</v>
+        <v>0.004506604506604228</v>
       </c>
       <c r="K45">
-        <v>1</v>
+        <v>0.9963775167658665</v>
       </c>
       <c r="L45">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="M45">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="46" spans="1:13">
       <c r="A46" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="B46" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C46">
         <v>3</v>
       </c>
       <c r="D46" t="s">
-        <v>122</v>
+        <v>109</v>
+      </c>
+      <c r="E46" t="s">
+        <v>105</v>
       </c>
       <c r="F46" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="G46">
-        <v>0.390625</v>
+        <v>0.109375</v>
       </c>
       <c r="H46">
-        <v>0.08745853842350808</v>
+        <v>0</v>
       </c>
       <c r="I46">
-        <v>0.693791461576492</v>
+        <v>0.2689246653106777</v>
       </c>
       <c r="J46">
-        <v>0.5053613053613053</v>
+        <v>0.006993006993006993</v>
       </c>
       <c r="K46">
-        <v>1</v>
+        <v>0.2447552447552448</v>
       </c>
       <c r="L46">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="M46">
-        <v>13</v>
+        <v>1422</v>
       </c>
     </row>
   </sheetData>
@@ -3113,7 +3137,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -3256,15 +3280,15 @@
         <v>157</v>
       </c>
       <c r="C13" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B14" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C14" t="s">
         <v>135</v>
@@ -3272,10 +3296,10 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B15" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C15" t="s">
         <v>135</v>
@@ -3283,10 +3307,10 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B16" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C16" t="s">
         <v>135</v>
@@ -3294,10 +3318,10 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B17" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C17" t="s">
         <v>135</v>
@@ -3305,10 +3329,10 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B18" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C18" t="s">
         <v>135</v>
@@ -3316,10 +3340,10 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B19" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C19" t="s">
         <v>135</v>
@@ -3327,10 +3351,10 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C20" t="s">
         <v>135</v>
@@ -3338,10 +3362,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B21" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C21" t="s">
         <v>135</v>
@@ -3349,10 +3373,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C22" t="s">
         <v>135</v>
@@ -3360,10 +3384,10 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B23" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C23" t="s">
         <v>135</v>
@@ -3371,10 +3395,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B24" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C24" t="s">
         <v>135</v>
@@ -3382,10 +3406,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B25" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C25" t="s">
         <v>135</v>
@@ -3393,13 +3417,13 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B26" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C26" t="s">
-        <v>184</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -3432,7 +3456,7 @@
         <v>190</v>
       </c>
       <c r="C29" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -3484,7 +3508,7 @@
         <v>199</v>
       </c>
       <c r="B34" t="s">
-        <v>147</v>
+        <v>200</v>
       </c>
       <c r="C34" t="s">
         <v>135</v>
@@ -3492,10 +3516,10 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B35" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C35" t="s">
         <v>135</v>
@@ -3503,10 +3527,10 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B36" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C36" t="s">
         <v>135</v>
@@ -3514,10 +3538,10 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B37" t="s">
-        <v>205</v>
+        <v>147</v>
       </c>
       <c r="C37" t="s">
         <v>135</v>
@@ -3542,6 +3566,50 @@
         <v>209</v>
       </c>
       <c r="C39" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>210</v>
+      </c>
+      <c r="B40" t="s">
+        <v>211</v>
+      </c>
+      <c r="C40" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>212</v>
+      </c>
+      <c r="B41" t="s">
+        <v>213</v>
+      </c>
+      <c r="C41" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>214</v>
+      </c>
+      <c r="B42" t="s">
+        <v>215</v>
+      </c>
+      <c r="C42" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>216</v>
+      </c>
+      <c r="B43" t="s">
+        <v>217</v>
+      </c>
+      <c r="C43" t="s">
         <v>135</v>
       </c>
     </row>

</xml_diff>